<commit_message>
1.7 Release + bug fixes
Released of 1.7 and some bug fixed, text mistaskes, minor bugs, etc.
</commit_message>
<xml_diff>
--- a/Count.xlsx
+++ b/Count.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2424" uniqueCount="397">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2524" uniqueCount="394">
   <si>
     <t>Gen 1</t>
   </si>
@@ -1203,16 +1203,878 @@
     <t>Energy Removal</t>
   </si>
   <si>
-    <t>R</t>
-  </si>
-  <si>
-    <t>G</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
     <t>Input</t>
   </si>
 </sst>
+</file>
+
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="9" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0070C0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+  </fonts>
+  <fills count="18">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0070C0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0066"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7030A0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.749992370372631"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1B7594"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.34998626667073579"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+  </fills>
+  <borders count="6">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+  </cellStyleXfs>
+  <cellXfs count="96">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="10" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="10" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+  </cellXfs>
+  <cellStyles count="2">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFF0066"/>
+      <color rgb="FF1B7594"/>
+    </mruColors>
+  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
+</styleSheet>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="0E2841"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E8E8E8"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="156082"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="E97132"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="196B24"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="0F9ED5"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="A02B93"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="4EA72E"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="467886"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="96607D"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
 </file>
</xml_diff>

<commit_message>
A new mechanic and bugs
</commit_message>
<xml_diff>
--- a/Count.xlsx
+++ b/Count.xlsx
@@ -2042,34 +2042,34 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">

</xml_diff>